<commit_message>
modified:   Analyst.xlsx modified:   __pycache__/data_analyzer.cpython-313.pyc modified:   data_analyzer.py modified:   flask_app.py new file:   static/Beartic.ico modified:   templates/index.html deleted:    templates/index.txt
</commit_message>
<xml_diff>
--- a/Analyst.xlsx
+++ b/Analyst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA0D2AD-341E-493A-A8EA-265E4542623E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5184F806-ED45-4B2E-910D-A002F745E922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -865,13 +865,22 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -890,15 +899,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1343,97 +1343,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="20" t="s">
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="O1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="19"/>
-      <c r="T1" s="19"/>
-      <c r="U1" s="19"/>
-      <c r="V1" s="19"/>
-      <c r="W1" s="19"/>
-      <c r="X1" s="19"/>
-      <c r="Y1" s="19"/>
-      <c r="Z1" s="20" t="s">
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="23"/>
+      <c r="T1" s="23"/>
+      <c r="U1" s="23"/>
+      <c r="V1" s="23"/>
+      <c r="W1" s="23"/>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
+      <c r="Z1" s="22" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="21" t="s">
+      <c r="A2" s="18"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="22" t="s">
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="22"/>
-      <c r="I2" s="23" t="s">
+      <c r="H2" s="25"/>
+      <c r="I2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="24" t="s">
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="24"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="25" t="s">
+      <c r="M2" s="27"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="22" t="s">
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="T2" s="22"/>
-      <c r="U2" s="26" t="s">
+      <c r="T2" s="25"/>
+      <c r="U2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="24" t="s">
+      <c r="V2" s="29"/>
+      <c r="W2" s="29"/>
+      <c r="X2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="Y2" s="24"/>
-      <c r="Z2" s="20"/>
+      <c r="Y2" s="27"/>
+      <c r="Z2" s="22"/>
     </row>
     <row r="3" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="18"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="20"/>
       <c r="D3" s="6" t="s">
         <v>10</v>
       </c>
@@ -1464,8 +1464,8 @@
       <c r="M3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="N3" s="20"/>
-      <c r="O3" s="18"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="20"/>
       <c r="P3" s="10" t="s">
         <v>10</v>
       </c>
@@ -1496,7 +1496,7 @@
       <c r="Y3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="Z3" s="20"/>
+      <c r="Z3" s="22"/>
     </row>
     <row r="4" spans="1:26" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -6623,11 +6623,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="16">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:M1"/>
-    <mergeCell ref="N1:N3"/>
     <mergeCell ref="O1:O3"/>
     <mergeCell ref="P1:Y1"/>
     <mergeCell ref="Z1:Z3"/>
@@ -6639,6 +6634,11 @@
     <mergeCell ref="S2:T2"/>
     <mergeCell ref="U2:W2"/>
     <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:M1"/>
+    <mergeCell ref="N1:N3"/>
   </mergeCells>
   <conditionalFormatting sqref="N1:N3">
     <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
@@ -6666,13 +6666,13 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:AMJ134"/>
+  <dimension ref="A1:AMI133"/>
   <sheetFormatPr defaultColWidth="12.69921875" defaultRowHeight="19.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1024" width="12.69921875" style="15"/>
+    <col min="1" max="1023" width="12.69921875" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>113</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>151</v>
       </c>
@@ -6721,23 +6721,22 @@
         <v>124</v>
       </c>
       <c r="F2" s="17">
-        <v>6.6</v>
+        <v>5.48</v>
       </c>
       <c r="G2" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H2" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I2" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J2" s="17">
-        <v>1</v>
-      </c>
-      <c r="K2" s="17"/>
-    </row>
-    <row r="3" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>185</v>
       </c>
@@ -6754,23 +6753,22 @@
         <v>141</v>
       </c>
       <c r="F3" s="17">
-        <v>9.1</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="G3" s="17">
-        <v>3.7</v>
+        <v>4.8899999999999997</v>
       </c>
       <c r="H3" s="17">
-        <v>7.5</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="I3" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J3" s="17">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="K3" s="17"/>
-    </row>
-    <row r="4" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>173</v>
       </c>
@@ -6787,23 +6785,22 @@
         <v>124</v>
       </c>
       <c r="F4" s="17">
-        <v>8</v>
+        <v>7.52</v>
       </c>
       <c r="G4" s="17">
-        <v>8.1</v>
+        <v>8.52</v>
       </c>
       <c r="H4" s="17">
-        <v>1.3</v>
+        <v>4.05</v>
       </c>
       <c r="I4" s="17">
-        <v>4.3</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="J4" s="17">
-        <v>5.2</v>
-      </c>
-      <c r="K4" s="17"/>
-    </row>
-    <row r="5" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>32</v>
       </c>
@@ -6820,23 +6817,22 @@
         <v>138</v>
       </c>
       <c r="F5" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.27</v>
       </c>
       <c r="G5" s="17">
-        <v>3.9</v>
+        <v>5.0599999999999996</v>
       </c>
       <c r="H5" s="17">
-        <v>5</v>
+        <v>7.02</v>
       </c>
       <c r="I5" s="17">
-        <v>4.0999999999999996</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="J5" s="17">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="K5" s="17"/>
-    </row>
-    <row r="6" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>174</v>
       </c>
@@ -6853,23 +6849,22 @@
         <v>158</v>
       </c>
       <c r="F6" s="17">
-        <v>7.9</v>
+        <v>7.38</v>
       </c>
       <c r="G6" s="17">
-        <v>7.6</v>
+        <v>8.11</v>
       </c>
       <c r="H6" s="17">
-        <v>4.0999999999999996</v>
+        <v>6.3</v>
       </c>
       <c r="I6" s="17">
         <v>3</v>
       </c>
       <c r="J6" s="17">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="K6" s="17"/>
-    </row>
-    <row r="7" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>167</v>
       </c>
@@ -6886,23 +6881,22 @@
         <v>124</v>
       </c>
       <c r="F7" s="17">
-        <v>7.3</v>
+        <v>6.5</v>
       </c>
       <c r="G7" s="17">
-        <v>8.5</v>
+        <v>8.85</v>
       </c>
       <c r="H7" s="17">
-        <v>0.8</v>
+        <v>3.64</v>
       </c>
       <c r="I7" s="17">
-        <v>4.8</v>
+        <v>4.88</v>
       </c>
       <c r="J7" s="17">
-        <v>2.6</v>
-      </c>
-      <c r="K7" s="17"/>
-    </row>
-    <row r="8" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.5599999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>187</v>
       </c>
@@ -6919,23 +6913,22 @@
         <v>129</v>
       </c>
       <c r="F8" s="17">
-        <v>5.7</v>
+        <v>4.17</v>
       </c>
       <c r="G8" s="17">
-        <v>3.5</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="H8" s="17">
-        <v>4.3</v>
+        <v>6.46</v>
       </c>
       <c r="I8" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J8" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K8" s="17"/>
-    </row>
-    <row r="9" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>156</v>
       </c>
@@ -6952,23 +6945,22 @@
         <v>138</v>
       </c>
       <c r="F9" s="17">
-        <v>6.9</v>
+        <v>5.92</v>
       </c>
       <c r="G9" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H9" s="17">
-        <v>1.2</v>
+        <v>3.97</v>
       </c>
       <c r="I9" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J9" s="17">
-        <v>6.2</v>
-      </c>
-      <c r="K9" s="17"/>
-    </row>
-    <row r="10" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.06</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>27</v>
       </c>
@@ -6985,23 +6977,22 @@
         <v>141</v>
       </c>
       <c r="F10" s="17">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="G10" s="17">
-        <v>7.7</v>
+        <v>8.19</v>
       </c>
       <c r="H10" s="17">
-        <v>6.5</v>
+        <v>8.23</v>
       </c>
       <c r="I10" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J10" s="17">
-        <v>3</v>
-      </c>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>195</v>
       </c>
@@ -7018,23 +7009,22 @@
         <v>124</v>
       </c>
       <c r="F11" s="17">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="G11" s="17">
-        <v>2.2000000000000002</v>
+        <v>3.66</v>
       </c>
       <c r="H11" s="17">
-        <v>7.5</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="I11" s="17">
-        <v>3.6</v>
+        <v>3.63</v>
       </c>
       <c r="J11" s="17">
-        <v>1.2</v>
-      </c>
-      <c r="K11" s="17"/>
-    </row>
-    <row r="12" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
         <v>159</v>
       </c>
@@ -7051,23 +7041,22 @@
         <v>124</v>
       </c>
       <c r="F12" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G12" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H12" s="17">
-        <v>0.8</v>
+        <v>3.64</v>
       </c>
       <c r="I12" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J12" s="17">
-        <v>2.6</v>
-      </c>
-      <c r="K12" s="17"/>
-    </row>
-    <row r="13" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.5599999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>143</v>
       </c>
@@ -7084,23 +7073,22 @@
         <v>124</v>
       </c>
       <c r="F13" s="17">
-        <v>5.7</v>
+        <v>4.17</v>
       </c>
       <c r="G13" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H13" s="17">
-        <v>6.3</v>
+        <v>8.07</v>
       </c>
       <c r="I13" s="17">
         <v>3</v>
       </c>
       <c r="J13" s="17">
-        <v>3</v>
-      </c>
-      <c r="K13" s="17"/>
-    </row>
-    <row r="14" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>86</v>
       </c>
@@ -7117,23 +7105,22 @@
         <v>158</v>
       </c>
       <c r="F14" s="17">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="G14" s="17">
-        <v>7.4</v>
+        <v>7.94</v>
       </c>
       <c r="H14" s="17">
-        <v>7</v>
+        <v>8.6300000000000008</v>
       </c>
       <c r="I14" s="17">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="J14" s="17">
-        <v>2.4</v>
-      </c>
-      <c r="K14" s="17"/>
-    </row>
-    <row r="15" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.3600000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>84</v>
       </c>
@@ -7150,23 +7137,22 @@
         <v>158</v>
       </c>
       <c r="F15" s="17">
-        <v>8</v>
+        <v>7.52</v>
       </c>
       <c r="G15" s="17">
-        <v>7.5</v>
+        <v>8.02</v>
       </c>
       <c r="H15" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I15" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J15" s="17">
-        <v>4.7</v>
-      </c>
-      <c r="K15" s="17"/>
-    </row>
-    <row r="16" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>160</v>
       </c>
@@ -7183,23 +7169,22 @@
         <v>125</v>
       </c>
       <c r="F16" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G16" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H16" s="17">
-        <v>4.2</v>
+        <v>6.38</v>
       </c>
       <c r="I16" s="17">
         <v>3</v>
       </c>
       <c r="J16" s="17">
-        <v>3.7</v>
-      </c>
-      <c r="K16" s="17"/>
-    </row>
-    <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>186</v>
       </c>
@@ -7216,23 +7201,22 @@
         <v>158</v>
       </c>
       <c r="F17" s="17">
-        <v>9.1</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="G17" s="17">
-        <v>3.8</v>
+        <v>4.9800000000000004</v>
       </c>
       <c r="H17" s="17">
-        <v>5.6</v>
+        <v>7.51</v>
       </c>
       <c r="I17" s="17">
         <v>3</v>
       </c>
       <c r="J17" s="17">
-        <v>3.2</v>
-      </c>
-      <c r="K17" s="17"/>
-    </row>
-    <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>23</v>
       </c>
@@ -7249,23 +7233,22 @@
         <v>141</v>
       </c>
       <c r="F18" s="17">
-        <v>9.6999999999999993</v>
+        <v>10</v>
       </c>
       <c r="G18" s="17">
-        <v>5.3</v>
+        <v>6.21</v>
       </c>
       <c r="H18" s="17">
-        <v>5.0999999999999996</v>
+        <v>7.1</v>
       </c>
       <c r="I18" s="17">
-        <v>4.7</v>
+        <v>4.78</v>
       </c>
       <c r="J18" s="17">
-        <v>1</v>
-      </c>
-      <c r="K18" s="17"/>
-    </row>
-    <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>134</v>
       </c>
@@ -7282,23 +7265,22 @@
         <v>124</v>
       </c>
       <c r="F19" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G19" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H19" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I19" s="17">
         <v>3</v>
       </c>
       <c r="J19" s="17">
-        <v>6.7</v>
-      </c>
-      <c r="K19" s="17"/>
-    </row>
-    <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.5399999999999991</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>94</v>
       </c>
@@ -7315,23 +7297,22 @@
         <v>138</v>
       </c>
       <c r="F20" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.27</v>
       </c>
       <c r="G20" s="17">
-        <v>3.1</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="H20" s="17">
-        <v>5.6</v>
+        <v>7.51</v>
       </c>
       <c r="I20" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J20" s="17">
-        <v>3.4</v>
-      </c>
-      <c r="K20" s="17"/>
-    </row>
-    <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
         <v>95</v>
       </c>
@@ -7348,23 +7329,22 @@
         <v>125</v>
       </c>
       <c r="F21" s="17">
-        <v>6.4</v>
+        <v>5.48</v>
       </c>
       <c r="G21" s="17">
-        <v>7.8</v>
+        <v>8.27</v>
       </c>
       <c r="H21" s="17">
-        <v>1.8</v>
+        <v>4.45</v>
       </c>
       <c r="I21" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.43</v>
       </c>
       <c r="J21" s="17">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="K21" s="17"/>
-    </row>
-    <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
         <v>96</v>
       </c>
@@ -7381,23 +7361,22 @@
         <v>124</v>
       </c>
       <c r="F22" s="17">
-        <v>5.4</v>
+        <v>3.73</v>
       </c>
       <c r="G22" s="17">
-        <v>9</v>
+        <v>9.26</v>
       </c>
       <c r="H22" s="17">
-        <v>1.5</v>
+        <v>4.21</v>
       </c>
       <c r="I22" s="17">
         <v>3</v>
       </c>
       <c r="J22" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K22" s="17"/>
-    </row>
-    <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
         <v>110</v>
       </c>
@@ -7414,23 +7393,22 @@
         <v>124</v>
       </c>
       <c r="F23" s="17">
-        <v>5.4</v>
+        <v>3.73</v>
       </c>
       <c r="G23" s="17">
-        <v>9</v>
+        <v>9.26</v>
       </c>
       <c r="H23" s="17">
-        <v>1.2</v>
+        <v>3.97</v>
       </c>
       <c r="I23" s="17">
         <v>3.1</v>
       </c>
       <c r="J23" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K23" s="17"/>
-    </row>
-    <row r="24" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>192</v>
       </c>
@@ -7447,23 +7425,22 @@
         <v>158</v>
       </c>
       <c r="F24" s="17">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="G24" s="17">
-        <v>3.4</v>
+        <v>4.6500000000000004</v>
       </c>
       <c r="H24" s="17">
-        <v>5.4</v>
+        <v>7.34</v>
       </c>
       <c r="I24" s="17">
-        <v>4.3</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="J24" s="17">
-        <v>2.8</v>
-      </c>
-      <c r="K24" s="17"/>
-    </row>
-    <row r="25" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>142</v>
       </c>
@@ -7480,23 +7457,22 @@
         <v>124</v>
       </c>
       <c r="F25" s="17">
-        <v>6.7</v>
+        <v>5.63</v>
       </c>
       <c r="G25" s="17">
-        <v>9</v>
+        <v>9.26</v>
       </c>
       <c r="H25" s="17">
-        <v>5.4</v>
+        <v>7.34</v>
       </c>
       <c r="I25" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J25" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K25" s="17"/>
-    </row>
-    <row r="26" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>144</v>
       </c>
@@ -7513,23 +7489,22 @@
         <v>124</v>
       </c>
       <c r="F26" s="17">
-        <v>5.6</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="G26" s="17">
-        <v>8.5</v>
+        <v>8.85</v>
       </c>
       <c r="H26" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I26" s="17">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="J26" s="17">
-        <v>5.8</v>
-      </c>
-      <c r="K26" s="17"/>
-    </row>
-    <row r="27" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
         <v>80</v>
       </c>
@@ -7546,23 +7521,22 @@
         <v>124</v>
       </c>
       <c r="F27" s="17">
-        <v>8.5</v>
+        <v>8.25</v>
       </c>
       <c r="G27" s="17">
-        <v>2</v>
+        <v>3.49</v>
       </c>
       <c r="H27" s="17">
-        <v>5.3</v>
+        <v>7.26</v>
       </c>
       <c r="I27" s="17">
-        <v>7.2</v>
+        <v>7.39</v>
       </c>
       <c r="J27" s="17">
-        <v>2</v>
-      </c>
-      <c r="K27" s="17"/>
-    </row>
-    <row r="28" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
         <v>48</v>
       </c>
@@ -7579,23 +7553,22 @@
         <v>158</v>
       </c>
       <c r="F28" s="17">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="G28" s="17">
-        <v>7.3</v>
+        <v>7.86</v>
       </c>
       <c r="H28" s="17">
-        <v>6.4</v>
+        <v>8.15</v>
       </c>
       <c r="I28" s="17">
-        <v>6.6</v>
+        <v>6.76</v>
       </c>
       <c r="J28" s="17">
-        <v>5</v>
-      </c>
-      <c r="K28" s="17"/>
-    </row>
-    <row r="29" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
         <v>81</v>
       </c>
@@ -7612,23 +7585,22 @@
         <v>125</v>
       </c>
       <c r="F29" s="17">
-        <v>7.8</v>
+        <v>7.23</v>
       </c>
       <c r="G29" s="17">
-        <v>7.5</v>
+        <v>8.02</v>
       </c>
       <c r="H29" s="17">
-        <v>4.8</v>
+        <v>6.86</v>
       </c>
       <c r="I29" s="17">
-        <v>3.9</v>
+        <v>3.94</v>
       </c>
       <c r="J29" s="17">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="K29" s="17"/>
-    </row>
-    <row r="30" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>49</v>
       </c>
@@ -7645,23 +7617,22 @@
         <v>124</v>
       </c>
       <c r="F30" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G30" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H30" s="17">
-        <v>0.8</v>
+        <v>3.64</v>
       </c>
       <c r="I30" s="17">
-        <v>7.2</v>
+        <v>7.39</v>
       </c>
       <c r="J30" s="17">
-        <v>8.1</v>
-      </c>
-      <c r="K30" s="17"/>
-    </row>
-    <row r="31" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
         <v>135</v>
       </c>
@@ -7678,23 +7649,22 @@
         <v>124</v>
       </c>
       <c r="F31" s="17">
-        <v>5.2</v>
+        <v>3.44</v>
       </c>
       <c r="G31" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H31" s="17">
-        <v>1.1000000000000001</v>
+        <v>3.89</v>
       </c>
       <c r="I31" s="17">
         <v>3</v>
       </c>
       <c r="J31" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K31" s="17"/>
-    </row>
-    <row r="32" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
         <v>145</v>
       </c>
@@ -7711,23 +7681,22 @@
         <v>124</v>
       </c>
       <c r="F32" s="17">
-        <v>5.7</v>
+        <v>4.17</v>
       </c>
       <c r="G32" s="17">
-        <v>8.5</v>
+        <v>8.85</v>
       </c>
       <c r="H32" s="17">
-        <v>3.6</v>
+        <v>5.9</v>
       </c>
       <c r="I32" s="17">
         <v>3</v>
       </c>
       <c r="J32" s="17">
-        <v>3.1</v>
-      </c>
-      <c r="K32" s="17"/>
-    </row>
-    <row r="33" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>188</v>
       </c>
@@ -7744,23 +7713,22 @@
         <v>124</v>
       </c>
       <c r="F33" s="17">
-        <v>5.0999999999999996</v>
+        <v>3.29</v>
       </c>
       <c r="G33" s="17">
-        <v>3.4</v>
+        <v>4.6500000000000004</v>
       </c>
       <c r="H33" s="17">
-        <v>4</v>
+        <v>6.22</v>
       </c>
       <c r="I33" s="17">
         <v>3</v>
       </c>
       <c r="J33" s="17">
-        <v>1.3</v>
-      </c>
-      <c r="K33" s="17"/>
-    </row>
-    <row r="34" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>175</v>
       </c>
@@ -7777,23 +7745,22 @@
         <v>138</v>
       </c>
       <c r="F34" s="17">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="G34" s="17">
-        <v>8</v>
+        <v>8.44</v>
       </c>
       <c r="H34" s="17">
-        <v>0.8</v>
+        <v>3.64</v>
       </c>
       <c r="I34" s="17">
-        <v>3.7</v>
+        <v>3.73</v>
       </c>
       <c r="J34" s="17">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="K34" s="17"/>
-    </row>
-    <row r="35" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
         <v>184</v>
       </c>
@@ -7810,23 +7777,22 @@
         <v>141</v>
       </c>
       <c r="F35" s="17">
-        <v>8.6999999999999993</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="G35" s="17">
-        <v>5.2</v>
+        <v>6.13</v>
       </c>
       <c r="H35" s="17">
-        <v>7.7</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="I35" s="17">
         <v>3</v>
       </c>
       <c r="J35" s="17">
-        <v>3.2</v>
-      </c>
-      <c r="K35" s="17"/>
-    </row>
-    <row r="36" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>65</v>
       </c>
@@ -7843,23 +7809,22 @@
         <v>125</v>
       </c>
       <c r="F36" s="17">
-        <v>8.9</v>
+        <v>8.83</v>
       </c>
       <c r="G36" s="17">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="H36" s="17">
-        <v>2.6</v>
+        <v>5.09</v>
       </c>
       <c r="I36" s="17">
-        <v>5.4</v>
+        <v>5.51</v>
       </c>
       <c r="J36" s="17">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="K36" s="17"/>
-    </row>
-    <row r="37" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>193</v>
       </c>
@@ -7876,23 +7841,22 @@
         <v>124</v>
       </c>
       <c r="F37" s="17">
-        <v>6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="G37" s="17">
-        <v>2.2000000000000002</v>
+        <v>3.66</v>
       </c>
       <c r="H37" s="17">
-        <v>1.2</v>
+        <v>3.97</v>
       </c>
       <c r="I37" s="17">
         <v>3</v>
       </c>
       <c r="J37" s="17">
-        <v>1</v>
-      </c>
-      <c r="K37" s="17"/>
-    </row>
-    <row r="38" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>146</v>
       </c>
@@ -7909,23 +7873,22 @@
         <v>124</v>
       </c>
       <c r="F38" s="17">
-        <v>5.4</v>
+        <v>3.73</v>
       </c>
       <c r="G38" s="17">
-        <v>8.6999999999999993</v>
+        <v>9.01</v>
       </c>
       <c r="H38" s="17">
-        <v>6.2</v>
+        <v>7.99</v>
       </c>
       <c r="I38" s="17">
         <v>3</v>
       </c>
       <c r="J38" s="17">
-        <v>3.1</v>
-      </c>
-      <c r="K38" s="17"/>
-    </row>
-    <row r="39" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>24</v>
       </c>
@@ -7942,23 +7905,22 @@
         <v>124</v>
       </c>
       <c r="F39" s="17">
-        <v>6.6</v>
+        <v>5.48</v>
       </c>
       <c r="G39" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H39" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I39" s="17">
-        <v>9.6999999999999993</v>
+        <v>10</v>
       </c>
       <c r="J39" s="17">
-        <v>7.6</v>
-      </c>
-      <c r="K39" s="17"/>
-    </row>
-    <row r="40" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9.42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
         <v>92</v>
       </c>
@@ -7975,23 +7937,22 @@
         <v>141</v>
       </c>
       <c r="F40" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G40" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H40" s="17">
-        <v>4.5999999999999996</v>
+        <v>6.7</v>
       </c>
       <c r="I40" s="17">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="J40" s="17">
-        <v>6</v>
-      </c>
-      <c r="K40" s="17"/>
-    </row>
-    <row r="41" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
         <v>194</v>
       </c>
@@ -8008,23 +7969,22 @@
         <v>124</v>
       </c>
       <c r="F41" s="17">
-        <v>5</v>
+        <v>3.15</v>
       </c>
       <c r="G41" s="17">
-        <v>2.2000000000000002</v>
+        <v>3.66</v>
       </c>
       <c r="H41" s="17">
-        <v>3</v>
+        <v>5.41</v>
       </c>
       <c r="I41" s="17">
         <v>3</v>
       </c>
       <c r="J41" s="17">
-        <v>1</v>
-      </c>
-      <c r="K41" s="17"/>
-    </row>
-    <row r="42" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>196</v>
       </c>
@@ -8041,23 +8001,22 @@
         <v>124</v>
       </c>
       <c r="F42" s="17">
-        <v>8.3000000000000007</v>
+        <v>7.96</v>
       </c>
       <c r="G42" s="17">
-        <v>3.5</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="H42" s="17">
-        <v>7</v>
+        <v>8.6300000000000008</v>
       </c>
       <c r="I42" s="17">
-        <v>3.6</v>
+        <v>3.63</v>
       </c>
       <c r="J42" s="17">
-        <v>1.3</v>
-      </c>
-      <c r="K42" s="17"/>
-    </row>
-    <row r="43" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
         <v>41</v>
       </c>
@@ -8074,23 +8033,22 @@
         <v>124</v>
       </c>
       <c r="F43" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.27</v>
       </c>
       <c r="G43" s="17">
-        <v>6.1</v>
+        <v>6.87</v>
       </c>
       <c r="H43" s="17">
-        <v>7.5</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="I43" s="17">
         <v>3</v>
       </c>
       <c r="J43" s="17">
-        <v>2.5</v>
-      </c>
-      <c r="K43" s="17"/>
-    </row>
-    <row r="44" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.46</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
         <v>37</v>
       </c>
@@ -8107,23 +8065,22 @@
         <v>158</v>
       </c>
       <c r="F44" s="17">
-        <v>7.9</v>
+        <v>7.38</v>
       </c>
       <c r="G44" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H44" s="17">
-        <v>4.5</v>
+        <v>6.62</v>
       </c>
       <c r="I44" s="17">
-        <v>5.4</v>
+        <v>5.51</v>
       </c>
       <c r="J44" s="17">
-        <v>7.8</v>
-      </c>
-      <c r="K44" s="17"/>
-    </row>
-    <row r="45" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9.61</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
         <v>57</v>
       </c>
@@ -8140,23 +8097,22 @@
         <v>158</v>
       </c>
       <c r="F45" s="17">
-        <v>9.3000000000000007</v>
+        <v>9.42</v>
       </c>
       <c r="G45" s="17">
-        <v>3.6</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="H45" s="17">
-        <v>7.2</v>
+        <v>8.7899999999999991</v>
       </c>
       <c r="I45" s="17">
         <v>3</v>
       </c>
       <c r="J45" s="17">
-        <v>3.6</v>
-      </c>
-      <c r="K45" s="17"/>
-    </row>
-    <row r="46" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
         <v>71</v>
       </c>
@@ -8173,23 +8129,22 @@
         <v>141</v>
       </c>
       <c r="F46" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.27</v>
       </c>
       <c r="G46" s="17">
-        <v>5</v>
+        <v>5.96</v>
       </c>
       <c r="H46" s="17">
-        <v>8.1999999999999993</v>
+        <v>9.6</v>
       </c>
       <c r="I46" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J46" s="17">
-        <v>3.3</v>
-      </c>
-      <c r="K46" s="17"/>
-    </row>
-    <row r="47" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
         <v>105</v>
       </c>
@@ -8206,23 +8161,22 @@
         <v>124</v>
       </c>
       <c r="F47" s="17">
-        <v>5.5</v>
+        <v>3.88</v>
       </c>
       <c r="G47" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H47" s="17">
-        <v>3.6</v>
+        <v>5.9</v>
       </c>
       <c r="I47" s="17">
         <v>3</v>
       </c>
       <c r="J47" s="17">
-        <v>3.8</v>
-      </c>
-      <c r="K47" s="17"/>
-    </row>
-    <row r="48" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>76</v>
       </c>
@@ -8239,23 +8193,22 @@
         <v>124</v>
       </c>
       <c r="F48" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G48" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H48" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I48" s="17">
-        <v>5.6</v>
+        <v>5.72</v>
       </c>
       <c r="J48" s="17">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="K48" s="17"/>
-    </row>
-    <row r="49" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
         <v>62</v>
       </c>
@@ -8272,23 +8225,22 @@
         <v>124</v>
       </c>
       <c r="F49" s="17">
-        <v>9.4</v>
+        <v>9.56</v>
       </c>
       <c r="G49" s="17">
-        <v>3.7</v>
+        <v>4.8899999999999997</v>
       </c>
       <c r="H49" s="17">
-        <v>8.6999999999999993</v>
+        <v>10</v>
       </c>
       <c r="I49" s="17">
         <v>3</v>
       </c>
       <c r="J49" s="17">
-        <v>3.1</v>
-      </c>
-      <c r="K49" s="17"/>
-    </row>
-    <row r="50" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
         <v>46</v>
       </c>
@@ -8305,23 +8257,22 @@
         <v>141</v>
       </c>
       <c r="F50" s="17">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="G50" s="17">
-        <v>7.5</v>
+        <v>8.02</v>
       </c>
       <c r="H50" s="17">
-        <v>6.3</v>
+        <v>8.07</v>
       </c>
       <c r="I50" s="17">
-        <v>5.7</v>
+        <v>5.82</v>
       </c>
       <c r="J50" s="17">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="K50" s="17"/>
-    </row>
-    <row r="51" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
         <v>152</v>
       </c>
@@ -8338,23 +8289,22 @@
         <v>129</v>
       </c>
       <c r="F51" s="17">
-        <v>6.6</v>
+        <v>5.48</v>
       </c>
       <c r="G51" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H51" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I51" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J51" s="17">
-        <v>1</v>
-      </c>
-      <c r="K51" s="17"/>
-    </row>
-    <row r="52" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
         <v>64</v>
       </c>
@@ -8371,23 +8321,22 @@
         <v>124</v>
       </c>
       <c r="F52" s="17">
-        <v>4.9000000000000004</v>
+        <v>3</v>
       </c>
       <c r="G52" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H52" s="17">
-        <v>2.2999999999999998</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="I52" s="17">
         <v>3</v>
       </c>
       <c r="J52" s="17">
-        <v>7.2</v>
-      </c>
-      <c r="K52" s="17"/>
-    </row>
-    <row r="53" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9.0299999999999994</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
         <v>153</v>
       </c>
@@ -8404,23 +8353,22 @@
         <v>124</v>
       </c>
       <c r="F53" s="17">
-        <v>6.4</v>
+        <v>5.19</v>
       </c>
       <c r="G53" s="17">
-        <v>8.6</v>
+        <v>8.93</v>
       </c>
       <c r="H53" s="17">
-        <v>3.1</v>
+        <v>5.49</v>
       </c>
       <c r="I53" s="17">
-        <v>5</v>
+        <v>5.09</v>
       </c>
       <c r="J53" s="17">
-        <v>3</v>
-      </c>
-      <c r="K53" s="17"/>
-    </row>
-    <row r="54" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>30</v>
       </c>
@@ -8437,23 +8385,22 @@
         <v>124</v>
       </c>
       <c r="F54" s="17">
-        <v>6.1</v>
+        <v>4.75</v>
       </c>
       <c r="G54" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H54" s="17">
-        <v>2.2999999999999998</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="I54" s="17">
-        <v>3.6</v>
+        <v>3.63</v>
       </c>
       <c r="J54" s="17">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="K54" s="17"/>
-    </row>
-    <row r="55" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="15" t="s">
         <v>63</v>
       </c>
@@ -8470,23 +8417,22 @@
         <v>124</v>
       </c>
       <c r="F55" s="17">
-        <v>6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="G55" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.42</v>
       </c>
       <c r="H55" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I55" s="17">
-        <v>7</v>
+        <v>7.18</v>
       </c>
       <c r="J55" s="17">
-        <v>1</v>
-      </c>
-      <c r="K55" s="17"/>
-    </row>
-    <row r="56" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
         <v>69</v>
       </c>
@@ -8503,23 +8449,22 @@
         <v>124</v>
       </c>
       <c r="F56" s="17">
-        <v>6.3</v>
+        <v>5.04</v>
       </c>
       <c r="G56" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H56" s="17">
-        <v>0.3</v>
+        <v>3.24</v>
       </c>
       <c r="I56" s="17">
-        <v>6</v>
+        <v>6.13</v>
       </c>
       <c r="J56" s="17">
-        <v>5.2</v>
-      </c>
-      <c r="K56" s="17"/>
-    </row>
-    <row r="57" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="15" t="s">
         <v>98</v>
       </c>
@@ -8536,23 +8481,22 @@
         <v>125</v>
       </c>
       <c r="F57" s="17">
-        <v>6.3</v>
+        <v>5.04</v>
       </c>
       <c r="G57" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H57" s="17">
-        <v>4.3</v>
+        <v>6.46</v>
       </c>
       <c r="I57" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J57" s="17">
-        <v>4</v>
-      </c>
-      <c r="K57" s="17"/>
-    </row>
-    <row r="58" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
         <v>25</v>
       </c>
@@ -8569,23 +8513,22 @@
         <v>158</v>
       </c>
       <c r="F58" s="17">
-        <v>9.1</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="G58" s="17">
-        <v>7.6</v>
+        <v>8.11</v>
       </c>
       <c r="H58" s="17">
-        <v>4</v>
+        <v>6.22</v>
       </c>
       <c r="I58" s="17">
-        <v>5.5</v>
+        <v>5.61</v>
       </c>
       <c r="J58" s="17">
-        <v>4.7</v>
-      </c>
-      <c r="K58" s="17"/>
-    </row>
-    <row r="59" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
         <v>59</v>
       </c>
@@ -8602,23 +8545,22 @@
         <v>124</v>
       </c>
       <c r="F59" s="17">
-        <v>9.4</v>
+        <v>9.56</v>
       </c>
       <c r="G59" s="17">
-        <v>3.1</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="H59" s="17">
-        <v>6</v>
+        <v>7.83</v>
       </c>
       <c r="I59" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J59" s="17">
-        <v>3.5</v>
-      </c>
-      <c r="K59" s="17"/>
-    </row>
-    <row r="60" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.43</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
         <v>130</v>
       </c>
@@ -8635,23 +8577,22 @@
         <v>124</v>
       </c>
       <c r="F60" s="17">
-        <v>5.0999999999999996</v>
+        <v>3.29</v>
       </c>
       <c r="G60" s="17">
-        <v>9.4</v>
+        <v>9.59</v>
       </c>
       <c r="H60" s="17">
-        <v>0.4</v>
+        <v>3.32</v>
       </c>
       <c r="I60" s="17">
-        <v>4.3</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="J60" s="17">
-        <v>5.2</v>
-      </c>
-      <c r="K60" s="17"/>
-    </row>
-    <row r="61" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
         <v>136</v>
       </c>
@@ -8668,23 +8609,22 @@
         <v>124</v>
       </c>
       <c r="F61" s="17">
-        <v>5</v>
+        <v>3.15</v>
       </c>
       <c r="G61" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H61" s="17">
-        <v>1.8</v>
+        <v>4.45</v>
       </c>
       <c r="I61" s="17">
         <v>3</v>
       </c>
       <c r="J61" s="17">
-        <v>5.6</v>
-      </c>
-      <c r="K61" s="17"/>
-    </row>
-    <row r="62" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.47</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
         <v>182</v>
       </c>
@@ -8701,23 +8641,22 @@
         <v>124</v>
       </c>
       <c r="F62" s="17">
-        <v>7.6</v>
+        <v>6.94</v>
       </c>
       <c r="G62" s="17">
-        <v>7.4</v>
+        <v>7.94</v>
       </c>
       <c r="H62" s="17">
-        <v>4.4000000000000004</v>
+        <v>6.54</v>
       </c>
       <c r="I62" s="17">
-        <v>3.8</v>
+        <v>3.84</v>
       </c>
       <c r="J62" s="17">
-        <v>3.1</v>
-      </c>
-      <c r="K62" s="17"/>
-    </row>
-    <row r="63" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
         <v>189</v>
       </c>
@@ -8734,23 +8673,22 @@
         <v>124</v>
       </c>
       <c r="F63" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.27</v>
       </c>
       <c r="G63" s="17">
-        <v>3.6</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="H63" s="17">
-        <v>6.5</v>
+        <v>8.23</v>
       </c>
       <c r="I63" s="17">
-        <v>4.8</v>
+        <v>4.88</v>
       </c>
       <c r="J63" s="17">
-        <v>1.4</v>
-      </c>
-      <c r="K63" s="17"/>
-    </row>
-    <row r="64" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.39</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
         <v>106</v>
       </c>
@@ -8767,23 +8705,22 @@
         <v>124</v>
       </c>
       <c r="F64" s="17">
-        <v>6.4</v>
+        <v>5.19</v>
       </c>
       <c r="G64" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.42</v>
       </c>
       <c r="H64" s="17">
-        <v>0.3</v>
+        <v>3.24</v>
       </c>
       <c r="I64" s="17">
-        <v>8</v>
+        <v>8.2200000000000006</v>
       </c>
       <c r="J64" s="17">
-        <v>6</v>
-      </c>
-      <c r="K64" s="17"/>
-    </row>
-    <row r="65" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="15" t="s">
         <v>161</v>
       </c>
@@ -8800,23 +8737,22 @@
         <v>124</v>
       </c>
       <c r="F65" s="17">
-        <v>6.5</v>
+        <v>5.33</v>
       </c>
       <c r="G65" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H65" s="17">
-        <v>5.5</v>
+        <v>7.43</v>
       </c>
       <c r="I65" s="17">
-        <v>4.4000000000000004</v>
+        <v>4.46</v>
       </c>
       <c r="J65" s="17">
-        <v>5.4</v>
-      </c>
-      <c r="K65" s="17"/>
-    </row>
-    <row r="66" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.28</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="15" t="s">
         <v>140</v>
       </c>
@@ -8833,23 +8769,22 @@
         <v>141</v>
       </c>
       <c r="F66" s="17">
-        <v>5.9</v>
+        <v>4.46</v>
       </c>
       <c r="G66" s="17">
-        <v>8.6</v>
+        <v>8.93</v>
       </c>
       <c r="H66" s="17">
-        <v>6.7</v>
+        <v>8.39</v>
       </c>
       <c r="I66" s="17">
-        <v>4.0999999999999996</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="J66" s="17">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="K66" s="17"/>
-    </row>
-    <row r="67" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.17</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="15" t="s">
         <v>154</v>
       </c>
@@ -8866,23 +8801,22 @@
         <v>124</v>
       </c>
       <c r="F67" s="17">
-        <v>5.8</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="G67" s="17">
-        <v>8.6999999999999993</v>
+        <v>9.01</v>
       </c>
       <c r="H67" s="17">
-        <v>4.2</v>
+        <v>6.38</v>
       </c>
       <c r="I67" s="17">
         <v>3</v>
       </c>
       <c r="J67" s="17">
-        <v>2</v>
-      </c>
-      <c r="K67" s="17"/>
-    </row>
-    <row r="68" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="15" t="s">
         <v>111</v>
       </c>
@@ -8899,23 +8833,22 @@
         <v>124</v>
       </c>
       <c r="F68" s="17">
-        <v>7.2</v>
+        <v>6.35</v>
       </c>
       <c r="G68" s="17">
-        <v>3.2</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="H68" s="17">
-        <v>5.0999999999999996</v>
+        <v>7.1</v>
       </c>
       <c r="I68" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J68" s="17">
-        <v>3</v>
-      </c>
-      <c r="K68" s="17"/>
-    </row>
-    <row r="69" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
         <v>38</v>
       </c>
@@ -8932,23 +8865,22 @@
         <v>124</v>
       </c>
       <c r="F69" s="17">
-        <v>7.1</v>
+        <v>6.21</v>
       </c>
       <c r="G69" s="17">
-        <v>3.6</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="H69" s="17">
-        <v>7.8</v>
+        <v>9.2799999999999994</v>
       </c>
       <c r="I69" s="17">
-        <v>6.6</v>
+        <v>6.76</v>
       </c>
       <c r="J69" s="17">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="K69" s="17"/>
-    </row>
-    <row r="70" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
         <v>170</v>
       </c>
@@ -8965,23 +8897,22 @@
         <v>124</v>
       </c>
       <c r="F70" s="17">
-        <v>6.6</v>
+        <v>5.48</v>
       </c>
       <c r="G70" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H70" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I70" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J70" s="17">
-        <v>1</v>
-      </c>
-      <c r="K70" s="17"/>
-    </row>
-    <row r="71" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
         <v>40</v>
       </c>
@@ -8998,23 +8929,22 @@
         <v>124</v>
       </c>
       <c r="F71" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G71" s="17">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="H71" s="17">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="I71" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J71" s="17">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="K71" s="17"/>
-    </row>
-    <row r="72" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.31</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
         <v>44</v>
       </c>
@@ -9031,23 +8961,22 @@
         <v>158</v>
       </c>
       <c r="F72" s="17">
-        <v>8.1</v>
+        <v>7.67</v>
       </c>
       <c r="G72" s="17">
-        <v>7.4</v>
+        <v>7.94</v>
       </c>
       <c r="H72" s="17">
-        <v>5.4</v>
+        <v>7.34</v>
       </c>
       <c r="I72" s="17">
-        <v>5.4</v>
+        <v>5.51</v>
       </c>
       <c r="J72" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K72" s="17"/>
-    </row>
-    <row r="73" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="15" t="s">
         <v>101</v>
       </c>
@@ -9064,23 +8993,22 @@
         <v>124</v>
       </c>
       <c r="F73" s="17">
-        <v>9.3000000000000007</v>
+        <v>9.42</v>
       </c>
       <c r="G73" s="17">
-        <v>3.5</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="H73" s="17">
-        <v>7.4</v>
+        <v>8.9499999999999993</v>
       </c>
       <c r="I73" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J73" s="17">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="K73" s="17"/>
-    </row>
-    <row r="74" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
         <v>53</v>
       </c>
@@ -9097,23 +9025,22 @@
         <v>125</v>
       </c>
       <c r="F74" s="17">
-        <v>5.2</v>
+        <v>3.44</v>
       </c>
       <c r="G74" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H74" s="17">
-        <v>4.8</v>
+        <v>6.86</v>
       </c>
       <c r="I74" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J74" s="17">
-        <v>5.5</v>
-      </c>
-      <c r="K74" s="17"/>
-    </row>
-    <row r="75" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.38</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="15" t="s">
         <v>70</v>
       </c>
@@ -9130,23 +9057,22 @@
         <v>124</v>
       </c>
       <c r="F75" s="17">
-        <v>6.5</v>
+        <v>5.33</v>
       </c>
       <c r="G75" s="17">
-        <v>7.6</v>
+        <v>8.11</v>
       </c>
       <c r="H75" s="17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I75" s="17">
-        <v>8</v>
+        <v>8.2200000000000006</v>
       </c>
       <c r="J75" s="17">
-        <v>7.1</v>
-      </c>
-      <c r="K75" s="17"/>
-    </row>
-    <row r="76" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.93</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
         <v>43</v>
       </c>
@@ -9163,23 +9089,22 @@
         <v>125</v>
       </c>
       <c r="F76" s="17">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="G76" s="17">
-        <v>7.4</v>
+        <v>7.94</v>
       </c>
       <c r="H76" s="17">
-        <v>4.2</v>
+        <v>6.38</v>
       </c>
       <c r="I76" s="17">
-        <v>3.5</v>
+        <v>3.52</v>
       </c>
       <c r="J76" s="17">
-        <v>3</v>
-      </c>
-      <c r="K76" s="17"/>
-    </row>
-    <row r="77" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="15" t="s">
         <v>131</v>
       </c>
@@ -9196,23 +9121,22 @@
         <v>124</v>
       </c>
       <c r="F77" s="17">
-        <v>4.9000000000000004</v>
+        <v>3</v>
       </c>
       <c r="G77" s="17">
-        <v>9.3000000000000007</v>
+        <v>9.51</v>
       </c>
       <c r="H77" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I77" s="17">
         <v>3</v>
       </c>
       <c r="J77" s="17">
-        <v>4.3</v>
-      </c>
-      <c r="K77" s="17"/>
-    </row>
-    <row r="78" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
         <v>36</v>
       </c>
@@ -9229,23 +9153,22 @@
         <v>124</v>
       </c>
       <c r="F78" s="17">
-        <v>8.1</v>
+        <v>7.67</v>
       </c>
       <c r="G78" s="17">
-        <v>7.9</v>
+        <v>8.35</v>
       </c>
       <c r="H78" s="17">
-        <v>4.7</v>
+        <v>6.78</v>
       </c>
       <c r="I78" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J78" s="17">
-        <v>5</v>
-      </c>
-      <c r="K78" s="17"/>
-    </row>
-    <row r="79" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.89</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
         <v>75</v>
       </c>
@@ -9262,23 +9185,22 @@
         <v>124</v>
       </c>
       <c r="F79" s="17">
-        <v>5</v>
+        <v>3.15</v>
       </c>
       <c r="G79" s="17">
-        <v>9.3000000000000007</v>
+        <v>9.51</v>
       </c>
       <c r="H79" s="17">
-        <v>2.1</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="I79" s="17">
         <v>3</v>
       </c>
       <c r="J79" s="17">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="K79" s="17"/>
-    </row>
-    <row r="80" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="15" t="s">
         <v>155</v>
       </c>
@@ -9295,23 +9217,22 @@
         <v>124</v>
       </c>
       <c r="F80" s="17">
-        <v>6.3</v>
+        <v>5.04</v>
       </c>
       <c r="G80" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H80" s="17">
-        <v>1.4</v>
+        <v>4.13</v>
       </c>
       <c r="I80" s="17">
-        <v>9</v>
+        <v>9.27</v>
       </c>
       <c r="J80" s="17">
-        <v>5</v>
-      </c>
-      <c r="K80" s="17"/>
-    </row>
-    <row r="81" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.89</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="15" t="s">
         <v>197</v>
       </c>
@@ -9328,23 +9249,22 @@
         <v>124</v>
       </c>
       <c r="F81" s="17">
-        <v>8.3000000000000007</v>
+        <v>7.96</v>
       </c>
       <c r="G81" s="17">
-        <v>1.4</v>
+        <v>3</v>
       </c>
       <c r="H81" s="17">
-        <v>5.0999999999999996</v>
+        <v>7.1</v>
       </c>
       <c r="I81" s="17">
         <v>3.1</v>
       </c>
       <c r="J81" s="17">
-        <v>1.4</v>
-      </c>
-      <c r="K81" s="17"/>
-    </row>
-    <row r="82" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.39</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="15" t="s">
         <v>104</v>
       </c>
@@ -9361,23 +9281,22 @@
         <v>138</v>
       </c>
       <c r="F82" s="17">
-        <v>8.1999999999999993</v>
+        <v>7.81</v>
       </c>
       <c r="G82" s="17">
-        <v>7.9</v>
+        <v>8.35</v>
       </c>
       <c r="H82" s="17">
-        <v>2.7</v>
+        <v>5.17</v>
       </c>
       <c r="I82" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J82" s="17">
-        <v>3.8</v>
-      </c>
-      <c r="K82" s="17"/>
-    </row>
-    <row r="83" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.72</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
         <v>87</v>
       </c>
@@ -9394,23 +9313,22 @@
         <v>125</v>
       </c>
       <c r="F83" s="17">
-        <v>6.6</v>
+        <v>5.48</v>
       </c>
       <c r="G83" s="17">
-        <v>9.4</v>
+        <v>9.59</v>
       </c>
       <c r="H83" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I83" s="17">
         <v>3</v>
       </c>
       <c r="J83" s="17">
-        <v>4.8</v>
-      </c>
-      <c r="K83" s="17"/>
-    </row>
-    <row r="84" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.69</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>67</v>
       </c>
@@ -9427,23 +9345,22 @@
         <v>124</v>
       </c>
       <c r="F84" s="17">
-        <v>5.8</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="G84" s="17">
-        <v>8.6999999999999993</v>
+        <v>9.01</v>
       </c>
       <c r="H84" s="17">
-        <v>6.1</v>
+        <v>7.91</v>
       </c>
       <c r="I84" s="17">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="J84" s="17">
-        <v>2.6</v>
-      </c>
-      <c r="K84" s="17"/>
-    </row>
-    <row r="85" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.5599999999999996</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="15" t="s">
         <v>82</v>
       </c>
@@ -9460,23 +9377,22 @@
         <v>124</v>
       </c>
       <c r="F85" s="17">
-        <v>6.2</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="G85" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H85" s="17">
-        <v>1.2</v>
+        <v>3.97</v>
       </c>
       <c r="I85" s="17">
         <v>3</v>
       </c>
       <c r="J85" s="17">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="K85" s="17"/>
-    </row>
-    <row r="86" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.31</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="15" t="s">
         <v>31</v>
       </c>
@@ -9493,23 +9409,22 @@
         <v>124</v>
       </c>
       <c r="F86" s="17">
-        <v>6.5</v>
+        <v>5.33</v>
       </c>
       <c r="G86" s="17">
-        <v>2.2999999999999998</v>
+        <v>3.74</v>
       </c>
       <c r="H86" s="17">
-        <v>7.6</v>
+        <v>9.11</v>
       </c>
       <c r="I86" s="17">
-        <v>5.8</v>
+        <v>5.93</v>
       </c>
       <c r="J86" s="17">
-        <v>1.3</v>
-      </c>
-      <c r="K86" s="17"/>
-    </row>
-    <row r="87" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="15" t="s">
         <v>176</v>
       </c>
@@ -9526,23 +9441,22 @@
         <v>158</v>
       </c>
       <c r="F87" s="17">
-        <v>7.9</v>
+        <v>7.38</v>
       </c>
       <c r="G87" s="17">
-        <v>7.4</v>
+        <v>7.94</v>
       </c>
       <c r="H87" s="17">
-        <v>5.2</v>
+        <v>7.18</v>
       </c>
       <c r="I87" s="17">
-        <v>3.5</v>
+        <v>3.52</v>
       </c>
       <c r="J87" s="17">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="K87" s="17"/>
-    </row>
-    <row r="88" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
         <v>99</v>
       </c>
@@ -9559,23 +9473,22 @@
         <v>125</v>
       </c>
       <c r="F88" s="17">
-        <v>8.8000000000000007</v>
+        <v>8.69</v>
       </c>
       <c r="G88" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H88" s="17">
-        <v>0.4</v>
+        <v>3.32</v>
       </c>
       <c r="I88" s="17">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="J88" s="17">
-        <v>3</v>
-      </c>
-      <c r="K88" s="17"/>
-    </row>
-    <row r="89" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.9400000000000004</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="15" t="s">
         <v>108</v>
       </c>
@@ -9592,23 +9505,22 @@
         <v>124</v>
       </c>
       <c r="F89" s="17">
-        <v>5.6</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="G89" s="17">
-        <v>3.8</v>
+        <v>4.9800000000000004</v>
       </c>
       <c r="H89" s="17">
-        <v>3.4</v>
+        <v>5.74</v>
       </c>
       <c r="I89" s="17">
-        <v>5.7</v>
+        <v>5.82</v>
       </c>
       <c r="J89" s="17">
-        <v>1</v>
-      </c>
-      <c r="K89" s="17"/>
-    </row>
-    <row r="90" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
         <v>132</v>
       </c>
@@ -9625,23 +9537,22 @@
         <v>124</v>
       </c>
       <c r="F90" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G90" s="17">
-        <v>9.1</v>
+        <v>9.34</v>
       </c>
       <c r="H90" s="17">
-        <v>0.4</v>
+        <v>3.32</v>
       </c>
       <c r="I90" s="17">
         <v>3</v>
       </c>
       <c r="J90" s="17">
-        <v>6.2</v>
-      </c>
-      <c r="K90" s="17"/>
-    </row>
-    <row r="91" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.06</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
         <v>198</v>
       </c>
@@ -9658,23 +9569,22 @@
         <v>124</v>
       </c>
       <c r="F91" s="17">
-        <v>8.6999999999999993</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="G91" s="17">
-        <v>3</v>
+        <v>4.32</v>
       </c>
       <c r="H91" s="17">
-        <v>8.1</v>
+        <v>9.52</v>
       </c>
       <c r="I91" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J91" s="17">
-        <v>2.1</v>
-      </c>
-      <c r="K91" s="17"/>
-    </row>
-    <row r="92" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.07</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="15" t="s">
         <v>162</v>
       </c>
@@ -9691,23 +9601,22 @@
         <v>158</v>
       </c>
       <c r="F92" s="17">
-        <v>7</v>
+        <v>6.06</v>
       </c>
       <c r="G92" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H92" s="17">
-        <v>5.0999999999999996</v>
+        <v>7.1</v>
       </c>
       <c r="I92" s="17">
         <v>3</v>
       </c>
       <c r="J92" s="17">
-        <v>4.5</v>
-      </c>
-      <c r="K92" s="17"/>
-    </row>
-    <row r="93" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="15" t="s">
         <v>133</v>
       </c>
@@ -9724,23 +9633,22 @@
         <v>124</v>
       </c>
       <c r="F93" s="17">
-        <v>5.2</v>
+        <v>3.44</v>
       </c>
       <c r="G93" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.42</v>
       </c>
       <c r="H93" s="17">
-        <v>1.3</v>
+        <v>4.05</v>
       </c>
       <c r="I93" s="17">
         <v>3</v>
       </c>
       <c r="J93" s="17">
-        <v>6.2</v>
-      </c>
-      <c r="K93" s="17"/>
-    </row>
-    <row r="94" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.06</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="15" t="s">
         <v>79</v>
       </c>
@@ -9757,23 +9665,22 @@
         <v>124</v>
       </c>
       <c r="F94" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G94" s="17">
-        <v>9.3000000000000007</v>
+        <v>9.51</v>
       </c>
       <c r="H94" s="17">
-        <v>3.4</v>
+        <v>5.74</v>
       </c>
       <c r="I94" s="17">
-        <v>4.5999999999999996</v>
+        <v>4.67</v>
       </c>
       <c r="J94" s="17">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="K94" s="17"/>
-    </row>
-    <row r="95" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
         <v>147</v>
       </c>
@@ -9790,23 +9697,22 @@
         <v>124</v>
       </c>
       <c r="F95" s="17">
-        <v>5.4</v>
+        <v>3.73</v>
       </c>
       <c r="G95" s="17">
-        <v>8.6</v>
+        <v>8.93</v>
       </c>
       <c r="H95" s="17">
-        <v>5.2</v>
+        <v>7.18</v>
       </c>
       <c r="I95" s="17">
         <v>3</v>
       </c>
       <c r="J95" s="17">
-        <v>3.3</v>
-      </c>
-      <c r="K95" s="17"/>
-    </row>
-    <row r="96" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.24</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
         <v>171</v>
       </c>
@@ -9823,23 +9729,22 @@
         <v>124</v>
       </c>
       <c r="F96" s="17">
-        <v>6.3</v>
+        <v>5.04</v>
       </c>
       <c r="G96" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H96" s="17">
-        <v>1.6</v>
+        <v>4.29</v>
       </c>
       <c r="I96" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J96" s="17">
-        <v>2</v>
-      </c>
-      <c r="K96" s="17"/>
-    </row>
-    <row r="97" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.97</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
         <v>127</v>
       </c>
@@ -9856,23 +9761,22 @@
         <v>124</v>
       </c>
       <c r="F97" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G97" s="17">
-        <v>9.6</v>
+        <v>9.75</v>
       </c>
       <c r="H97" s="17">
-        <v>2.7</v>
+        <v>5.17</v>
       </c>
       <c r="I97" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J97" s="17">
-        <v>7</v>
-      </c>
-      <c r="K97" s="17"/>
-    </row>
-    <row r="98" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.83</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="15" t="s">
         <v>66</v>
       </c>
@@ -9889,23 +9793,22 @@
         <v>124</v>
       </c>
       <c r="F98" s="17">
-        <v>6.4</v>
+        <v>5.19</v>
       </c>
       <c r="G98" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H98" s="17">
-        <v>0.3</v>
+        <v>3.24</v>
       </c>
       <c r="I98" s="17">
-        <v>8</v>
+        <v>8.2200000000000006</v>
       </c>
       <c r="J98" s="17">
-        <v>1</v>
-      </c>
-      <c r="K98" s="17"/>
-    </row>
-    <row r="99" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="15" t="s">
         <v>148</v>
       </c>
@@ -9922,23 +9825,22 @@
         <v>124</v>
       </c>
       <c r="F99" s="17">
-        <v>5.5</v>
+        <v>3.88</v>
       </c>
       <c r="G99" s="17">
-        <v>8.5</v>
+        <v>8.85</v>
       </c>
       <c r="H99" s="17">
-        <v>1.5</v>
+        <v>4.21</v>
       </c>
       <c r="I99" s="17">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="J99" s="17">
-        <v>4.3</v>
-      </c>
-      <c r="K99" s="17"/>
-    </row>
-    <row r="100" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.21</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="15" t="s">
         <v>85</v>
       </c>
@@ -9955,23 +9857,22 @@
         <v>124</v>
       </c>
       <c r="F100" s="17">
-        <v>5.2</v>
+        <v>3.44</v>
       </c>
       <c r="G100" s="17">
-        <v>9</v>
+        <v>9.26</v>
       </c>
       <c r="H100" s="17">
-        <v>3.2</v>
+        <v>5.57</v>
       </c>
       <c r="I100" s="17">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="J100" s="17">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="K100" s="17"/>
-    </row>
-    <row r="101" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.01</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="15" t="s">
         <v>149</v>
       </c>
@@ -9988,23 +9889,22 @@
         <v>124</v>
       </c>
       <c r="F101" s="17">
-        <v>5.4</v>
+        <v>3.73</v>
       </c>
       <c r="G101" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H101" s="17">
-        <v>2.8</v>
+        <v>5.25</v>
       </c>
       <c r="I101" s="17">
         <v>3</v>
       </c>
       <c r="J101" s="17">
-        <v>3.2</v>
-      </c>
-      <c r="K101" s="17"/>
-    </row>
-    <row r="102" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="15" t="s">
         <v>169</v>
       </c>
@@ -10021,23 +9921,22 @@
         <v>158</v>
       </c>
       <c r="F102" s="17">
-        <v>7.2</v>
+        <v>6.35</v>
       </c>
       <c r="G102" s="17">
-        <v>8.4</v>
+        <v>8.76</v>
       </c>
       <c r="H102" s="17">
-        <v>3.2</v>
+        <v>5.57</v>
       </c>
       <c r="I102" s="17">
-        <v>6.8</v>
+        <v>6.97</v>
       </c>
       <c r="J102" s="17">
-        <v>8</v>
-      </c>
-      <c r="K102" s="17"/>
-    </row>
-    <row r="103" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="15" t="s">
         <v>58</v>
       </c>
@@ -10054,23 +9953,22 @@
         <v>124</v>
       </c>
       <c r="F103" s="17">
-        <v>6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="G103" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H103" s="17">
-        <v>3.9</v>
+        <v>6.14</v>
       </c>
       <c r="I103" s="17">
-        <v>4.4000000000000004</v>
+        <v>4.46</v>
       </c>
       <c r="J103" s="17">
-        <v>6.1</v>
-      </c>
-      <c r="K103" s="17"/>
-    </row>
-    <row r="104" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="15" t="s">
         <v>26</v>
       </c>
@@ -10087,23 +9985,22 @@
         <v>124</v>
       </c>
       <c r="F104" s="17">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="G104" s="17">
-        <v>7.3</v>
+        <v>7.86</v>
       </c>
       <c r="H104" s="17">
-        <v>5.7</v>
+        <v>7.59</v>
       </c>
       <c r="I104" s="17">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="J104" s="17">
-        <v>2.4</v>
-      </c>
-      <c r="K104" s="17"/>
-    </row>
-    <row r="105" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.3600000000000003</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="15" t="s">
         <v>137</v>
       </c>
@@ -10120,23 +10017,22 @@
         <v>125</v>
       </c>
       <c r="F105" s="17">
-        <v>5.3</v>
+        <v>3.58</v>
       </c>
       <c r="G105" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H105" s="17">
-        <v>3.3</v>
+        <v>5.66</v>
       </c>
       <c r="I105" s="17">
         <v>3</v>
       </c>
       <c r="J105" s="17">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="K105" s="17"/>
-    </row>
-    <row r="106" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="15" t="s">
         <v>190</v>
       </c>
@@ -10153,23 +10049,22 @@
         <v>124</v>
       </c>
       <c r="F106" s="17">
-        <v>5.8</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="G106" s="17">
-        <v>3.6</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="H106" s="17">
-        <v>4.0999999999999996</v>
+        <v>6.3</v>
       </c>
       <c r="I106" s="17">
-        <v>4.5999999999999996</v>
+        <v>4.67</v>
       </c>
       <c r="J106" s="17">
-        <v>2.6</v>
-      </c>
-      <c r="K106" s="17"/>
-    </row>
-    <row r="107" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.5599999999999996</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="15" t="s">
         <v>163</v>
       </c>
@@ -10186,23 +10081,22 @@
         <v>125</v>
       </c>
       <c r="F107" s="17">
-        <v>7</v>
+        <v>6.06</v>
       </c>
       <c r="G107" s="17">
-        <v>7.8</v>
+        <v>8.27</v>
       </c>
       <c r="H107" s="17">
-        <v>0.2</v>
+        <v>3.16</v>
       </c>
       <c r="I107" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J107" s="17">
-        <v>3.1</v>
-      </c>
-      <c r="K107" s="17"/>
-    </row>
-    <row r="108" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="15" t="s">
         <v>183</v>
       </c>
@@ -10219,23 +10113,22 @@
         <v>125</v>
       </c>
       <c r="F108" s="17">
-        <v>8.1</v>
+        <v>7.67</v>
       </c>
       <c r="G108" s="17">
-        <v>7.6</v>
+        <v>8.11</v>
       </c>
       <c r="H108" s="17">
-        <v>7.6</v>
+        <v>9.11</v>
       </c>
       <c r="I108" s="17">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="J108" s="17">
-        <v>3.6</v>
-      </c>
-      <c r="K108" s="17"/>
-    </row>
-    <row r="109" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="15" t="s">
         <v>172</v>
       </c>
@@ -10252,23 +10145,22 @@
         <v>124</v>
       </c>
       <c r="F109" s="17">
-        <v>6.3</v>
+        <v>5.04</v>
       </c>
       <c r="G109" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H109" s="17">
-        <v>1.2</v>
+        <v>3.97</v>
       </c>
       <c r="I109" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J109" s="17">
-        <v>1</v>
-      </c>
-      <c r="K109" s="17"/>
-    </row>
-    <row r="110" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="15" t="s">
         <v>102</v>
       </c>
@@ -10285,23 +10177,22 @@
         <v>141</v>
       </c>
       <c r="F110" s="17">
-        <v>5.9</v>
+        <v>4.46</v>
       </c>
       <c r="G110" s="17">
-        <v>8</v>
+        <v>8.44</v>
       </c>
       <c r="H110" s="17">
-        <v>2.5</v>
+        <v>5.01</v>
       </c>
       <c r="I110" s="17">
-        <v>6</v>
+        <v>6.13</v>
       </c>
       <c r="J110" s="17">
-        <v>4</v>
-      </c>
-      <c r="K110" s="17"/>
-    </row>
-    <row r="111" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="15" t="s">
         <v>177</v>
       </c>
@@ -10318,23 +10209,22 @@
         <v>125</v>
       </c>
       <c r="F111" s="17">
-        <v>7.9</v>
+        <v>7.38</v>
       </c>
       <c r="G111" s="17">
-        <v>7.8</v>
+        <v>8.27</v>
       </c>
       <c r="H111" s="17">
-        <v>4</v>
+        <v>6.22</v>
       </c>
       <c r="I111" s="17">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="J111" s="17">
-        <v>3.2</v>
-      </c>
-      <c r="K111" s="17"/>
-    </row>
-    <row r="112" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.14</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="15" t="s">
         <v>39</v>
       </c>
@@ -10351,23 +10241,22 @@
         <v>125</v>
       </c>
       <c r="F112" s="17">
-        <v>8.3000000000000007</v>
+        <v>7.96</v>
       </c>
       <c r="G112" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H112" s="17">
-        <v>6.6</v>
+        <v>8.31</v>
       </c>
       <c r="I112" s="17">
-        <v>4</v>
+        <v>4.04</v>
       </c>
       <c r="J112" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K112" s="17"/>
-    </row>
-    <row r="113" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="15" t="s">
         <v>178</v>
       </c>
@@ -10384,23 +10273,22 @@
         <v>124</v>
       </c>
       <c r="F113" s="17">
-        <v>7.4</v>
+        <v>6.65</v>
       </c>
       <c r="G113" s="17">
-        <v>8.6999999999999993</v>
+        <v>9.01</v>
       </c>
       <c r="H113" s="17">
-        <v>1.4</v>
+        <v>4.13</v>
       </c>
       <c r="I113" s="17">
-        <v>4.8</v>
+        <v>4.88</v>
       </c>
       <c r="J113" s="17">
-        <v>6.4</v>
-      </c>
-      <c r="K113" s="17"/>
-    </row>
-    <row r="114" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8.25</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="15" t="s">
         <v>29</v>
       </c>
@@ -10417,23 +10305,22 @@
         <v>158</v>
       </c>
       <c r="F114" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G114" s="17">
-        <v>7.7</v>
+        <v>8.19</v>
       </c>
       <c r="H114" s="17">
-        <v>1.5</v>
+        <v>4.21</v>
       </c>
       <c r="I114" s="17">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="J114" s="17">
-        <v>5.3</v>
-      </c>
-      <c r="K114" s="17"/>
-    </row>
-    <row r="115" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.18</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="15" t="s">
         <v>50</v>
       </c>
@@ -10450,23 +10337,22 @@
         <v>124</v>
       </c>
       <c r="F115" s="17">
-        <v>9</v>
+        <v>8.98</v>
       </c>
       <c r="G115" s="17">
-        <v>7.3</v>
+        <v>7.86</v>
       </c>
       <c r="H115" s="17">
-        <v>5.5</v>
+        <v>7.43</v>
       </c>
       <c r="I115" s="17">
         <v>3</v>
       </c>
       <c r="J115" s="17">
-        <v>4</v>
-      </c>
-      <c r="K115" s="17"/>
-    </row>
-    <row r="116" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="15" t="s">
         <v>180</v>
       </c>
@@ -10483,23 +10369,22 @@
         <v>125</v>
       </c>
       <c r="F116" s="17">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="G116" s="17">
-        <v>7.5</v>
+        <v>8.02</v>
       </c>
       <c r="H116" s="17">
-        <v>1.3</v>
+        <v>4.05</v>
       </c>
       <c r="I116" s="17">
-        <v>3.7</v>
+        <v>3.73</v>
       </c>
       <c r="J116" s="17">
-        <v>6</v>
-      </c>
-      <c r="K116" s="17"/>
-    </row>
-    <row r="117" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="15" t="s">
         <v>199</v>
       </c>
@@ -10516,23 +10401,22 @@
         <v>124</v>
       </c>
       <c r="F117" s="17">
-        <v>9.1</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="G117" s="17">
-        <v>2.4</v>
+        <v>3.82</v>
       </c>
       <c r="H117" s="17">
-        <v>7.3</v>
+        <v>8.8699999999999992</v>
       </c>
       <c r="I117" s="17">
         <v>3</v>
       </c>
       <c r="J117" s="17">
-        <v>1.6</v>
-      </c>
-      <c r="K117" s="17"/>
-    </row>
-    <row r="118" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="15" t="s">
         <v>55</v>
       </c>
@@ -10549,23 +10433,22 @@
         <v>138</v>
       </c>
       <c r="F118" s="17">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="G118" s="17">
-        <v>5.2</v>
+        <v>6.13</v>
       </c>
       <c r="H118" s="17">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="I118" s="17">
-        <v>5.7</v>
+        <v>5.82</v>
       </c>
       <c r="J118" s="17">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="K118" s="17"/>
-    </row>
-    <row r="119" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="15" t="s">
         <v>150</v>
       </c>
@@ -10582,23 +10465,22 @@
         <v>124</v>
       </c>
       <c r="F119" s="17">
-        <v>5.5</v>
+        <v>3.88</v>
       </c>
       <c r="G119" s="17">
-        <v>8.6</v>
+        <v>8.93</v>
       </c>
       <c r="H119" s="17">
-        <v>5.4</v>
+        <v>7.34</v>
       </c>
       <c r="I119" s="17">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="J119" s="17">
-        <v>2.7</v>
-      </c>
-      <c r="K119" s="17"/>
-    </row>
-    <row r="120" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.6500000000000004</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="15" t="s">
         <v>28</v>
       </c>
@@ -10615,23 +10497,22 @@
         <v>124</v>
       </c>
       <c r="F120" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G120" s="17">
-        <v>8.6</v>
+        <v>8.93</v>
       </c>
       <c r="H120" s="17">
-        <v>5.3</v>
+        <v>7.26</v>
       </c>
       <c r="I120" s="17">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="J120" s="17">
-        <v>3.4</v>
-      </c>
-      <c r="K120" s="17"/>
-    </row>
-    <row r="121" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.33</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="15" t="s">
         <v>72</v>
       </c>
@@ -10648,23 +10529,22 @@
         <v>124</v>
       </c>
       <c r="F121" s="17">
-        <v>6.2</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="G121" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H121" s="17">
-        <v>6.3</v>
+        <v>8.07</v>
       </c>
       <c r="I121" s="17">
         <v>3</v>
       </c>
       <c r="J121" s="17">
-        <v>3.6</v>
-      </c>
-      <c r="K121" s="17"/>
-    </row>
-    <row r="122" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="15" t="s">
         <v>77</v>
       </c>
@@ -10681,23 +10561,22 @@
         <v>124</v>
       </c>
       <c r="F122" s="17">
-        <v>5.6</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="G122" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H122" s="17">
-        <v>6</v>
+        <v>7.83</v>
       </c>
       <c r="I122" s="17">
         <v>3</v>
       </c>
       <c r="J122" s="17">
-        <v>5.9</v>
-      </c>
-      <c r="K122" s="17"/>
-    </row>
-    <row r="123" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.76</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="15" t="s">
         <v>112</v>
       </c>
@@ -10714,23 +10593,22 @@
         <v>124</v>
       </c>
       <c r="F123" s="17">
-        <v>5.0999999999999996</v>
+        <v>3.29</v>
       </c>
       <c r="G123" s="17">
-        <v>8.9</v>
+        <v>9.18</v>
       </c>
       <c r="H123" s="17">
-        <v>2.1</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="I123" s="17">
-        <v>5.6</v>
+        <v>5.72</v>
       </c>
       <c r="J123" s="17">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="K123" s="17"/>
-    </row>
-    <row r="124" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="15" t="s">
         <v>179</v>
       </c>
@@ -10747,23 +10625,22 @@
         <v>125</v>
       </c>
       <c r="F124" s="17">
-        <v>8.1</v>
+        <v>7.67</v>
       </c>
       <c r="G124" s="17">
-        <v>7.5</v>
+        <v>8.02</v>
       </c>
       <c r="H124" s="17">
-        <v>2.2000000000000002</v>
+        <v>4.7699999999999996</v>
       </c>
       <c r="I124" s="17">
         <v>3</v>
       </c>
       <c r="J124" s="17">
-        <v>4.2</v>
-      </c>
-      <c r="K124" s="17"/>
-    </row>
-    <row r="125" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.11</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="15" t="s">
         <v>139</v>
       </c>
@@ -10780,23 +10657,22 @@
         <v>124</v>
       </c>
       <c r="F125" s="17">
-        <v>5.8</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="G125" s="17">
-        <v>9</v>
+        <v>9.26</v>
       </c>
       <c r="H125" s="17">
-        <v>5.3</v>
+        <v>7.26</v>
       </c>
       <c r="I125" s="17">
         <v>3</v>
       </c>
       <c r="J125" s="17">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="K125" s="17"/>
-    </row>
-    <row r="126" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.79</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="15" t="s">
         <v>73</v>
       </c>
@@ -10813,23 +10689,22 @@
         <v>125</v>
       </c>
       <c r="F126" s="17">
-        <v>6.1</v>
+        <v>4.75</v>
       </c>
       <c r="G126" s="17">
-        <v>8.6999999999999993</v>
+        <v>9.01</v>
       </c>
       <c r="H126" s="17">
-        <v>4.9000000000000004</v>
+        <v>6.94</v>
       </c>
       <c r="I126" s="17">
-        <v>5.4</v>
+        <v>5.51</v>
       </c>
       <c r="J126" s="17">
-        <v>6.1</v>
-      </c>
-      <c r="K126" s="17"/>
-    </row>
-    <row r="127" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="15" t="s">
         <v>164</v>
       </c>
@@ -10846,23 +10721,22 @@
         <v>124</v>
       </c>
       <c r="F127" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G127" s="17">
-        <v>8.3000000000000007</v>
+        <v>8.68</v>
       </c>
       <c r="H127" s="17">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="I127" s="17">
-        <v>3.8</v>
+        <v>3.84</v>
       </c>
       <c r="J127" s="17">
-        <v>2.4</v>
-      </c>
-      <c r="K127" s="17"/>
-    </row>
-    <row r="128" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.3600000000000003</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="15" t="s">
         <v>68</v>
       </c>
@@ -10879,23 +10753,22 @@
         <v>124</v>
       </c>
       <c r="F128" s="17">
-        <v>7.8</v>
+        <v>7.23</v>
       </c>
       <c r="G128" s="17">
-        <v>7.7</v>
+        <v>8.19</v>
       </c>
       <c r="H128" s="17">
-        <v>5.2</v>
+        <v>7.18</v>
       </c>
       <c r="I128" s="17">
-        <v>3.3</v>
+        <v>3.31</v>
       </c>
       <c r="J128" s="17">
-        <v>3.6</v>
-      </c>
-      <c r="K128" s="17"/>
-    </row>
-    <row r="129" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="15" t="s">
         <v>42</v>
       </c>
@@ -10912,23 +10785,22 @@
         <v>124</v>
       </c>
       <c r="F129" s="17">
-        <v>6.4</v>
+        <v>5.19</v>
       </c>
       <c r="G129" s="17">
-        <v>8.5</v>
+        <v>8.85</v>
       </c>
       <c r="H129" s="17">
-        <v>6.2</v>
+        <v>7.99</v>
       </c>
       <c r="I129" s="17">
         <v>3</v>
       </c>
       <c r="J129" s="17">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="K129" s="17"/>
-    </row>
-    <row r="130" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="15" t="s">
         <v>47</v>
       </c>
@@ -10945,23 +10817,22 @@
         <v>124</v>
       </c>
       <c r="F130" s="17">
-        <v>6.1</v>
+        <v>4.75</v>
       </c>
       <c r="G130" s="17">
-        <v>8.8000000000000007</v>
+        <v>9.09</v>
       </c>
       <c r="H130" s="17">
-        <v>5.6</v>
+        <v>7.51</v>
       </c>
       <c r="I130" s="17">
         <v>3</v>
       </c>
       <c r="J130" s="17">
-        <v>5.2</v>
-      </c>
-      <c r="K130" s="17"/>
-    </row>
-    <row r="131" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="15" t="s">
         <v>165</v>
       </c>
@@ -10978,23 +10849,22 @@
         <v>124</v>
       </c>
       <c r="F131" s="17">
-        <v>5.7</v>
+        <v>4.17</v>
       </c>
       <c r="G131" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.42</v>
       </c>
       <c r="H131" s="17">
-        <v>3.1</v>
+        <v>5.49</v>
       </c>
       <c r="I131" s="17">
         <v>3</v>
       </c>
       <c r="J131" s="17">
-        <v>2.1</v>
-      </c>
-      <c r="K131" s="17"/>
-    </row>
-    <row r="132" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.07</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="15" t="s">
         <v>35</v>
       </c>
@@ -11011,23 +10881,22 @@
         <v>124</v>
       </c>
       <c r="F132" s="17">
-        <v>6.8</v>
+        <v>5.77</v>
       </c>
       <c r="G132" s="17">
-        <v>8.1999999999999993</v>
+        <v>8.6</v>
       </c>
       <c r="H132" s="17">
-        <v>7.2</v>
+        <v>8.7899999999999991</v>
       </c>
       <c r="I132" s="17">
         <v>3</v>
       </c>
       <c r="J132" s="17">
-        <v>4</v>
-      </c>
-      <c r="K132" s="17"/>
-    </row>
-    <row r="133" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="15" t="s">
         <v>166</v>
       </c>
@@ -11044,24 +10913,20 @@
         <v>124</v>
       </c>
       <c r="F133" s="17">
-        <v>6.5</v>
+        <v>5.33</v>
       </c>
       <c r="G133" s="17">
-        <v>9.1999999999999993</v>
+        <v>9.42</v>
       </c>
       <c r="H133" s="17">
-        <v>3.1</v>
+        <v>5.49</v>
       </c>
       <c r="I133" s="17">
-        <v>4.9000000000000004</v>
+        <v>4.99</v>
       </c>
       <c r="J133" s="17">
-        <v>7.2</v>
-      </c>
-      <c r="K133" s="17"/>
-    </row>
-    <row r="134" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K134" s="17"/>
+        <v>9.0299999999999994</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J133" xr:uid="{00000000-0001-0000-0100-000000000000}">

</xml_diff>